<commit_message>
Unify PE/PB median for HPG valuation snapshot with the Excel-matching source
peMedian/pbMedian (used in the web's valuation snapshot card, e.g. "P/E Muc tieu") were computed
from a separate flat median across all quarters, diverging from PE_HIST_MEDIAN/PB_HIST_MEDIAN
(the median-of-yearly-medians already used for the actual target price and shown in Excel/PDF).
This caused the web to show 9.7x while PDF/Excel showed 10.3x for the same "P/E" concept - now
both read from the single shared source.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/HPG/HPG_Model_2026_07_03.xlsx
+++ b/Bao cao/HPG/HPG_Model_2026_07_03.xlsx
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>03/07/2026 15:44</t>
+          <t>03/07/2026 18:03</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="B31" s="35" t="inlineStr">
         <is>
-          <t>+12,715 tỷ</t>
+          <t>+12,720 tỷ</t>
         </is>
       </c>
       <c r="C31" s="74" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="B33" s="35" t="inlineStr">
         <is>
-          <t>168,831 tỷ</t>
+          <t>168,836 tỷ</t>
         </is>
       </c>
       <c r="C33" s="74" t="inlineStr">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="B41" s="35" t="inlineStr">
         <is>
-          <t>+5,395 tỷ</t>
+          <t>+5,396 tỷ</t>
         </is>
       </c>
       <c r="C41" s="74" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="B43" s="35" t="inlineStr">
         <is>
-          <t>20,848 tỷ</t>
+          <t>20,849 tỷ</t>
         </is>
       </c>
       <c r="C43" s="74" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="C43" s="35" t="inlineStr">
         <is>
-          <t>KH 2026E NI: 20,848 tỷ</t>
+          <t>KH 2026E NI: 20,849 tỷ</t>
         </is>
       </c>
       <c r="D43" s="35" t="inlineStr">
@@ -13178,7 +13178,7 @@
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>564.6</v>
+        <v>564.5</v>
       </c>
       <c r="H21" s="108" t="inlineStr">
         <is>
@@ -13227,7 +13227,7 @@
         </is>
       </c>
       <c r="G22" s="10" t="n">
-        <v>585.7</v>
+        <v>585.6</v>
       </c>
       <c r="H22" s="108" t="inlineStr">
         <is>
@@ -13278,7 +13278,7 @@
       </c>
       <c r="H25" s="94" t="inlineStr">
         <is>
-          <t>SteelOnline noi dia (15,120 dong/kg, quy doi ty gia 26,295)</t>
+          <t>SteelOnline noi dia (15,120 dong/kg, quy doi ty gia 26,296)</t>
         </is>
       </c>
     </row>
@@ -14791,13 +14791,13 @@
         <v>26000</v>
       </c>
       <c r="G25" s="10" t="n">
-        <v>26295</v>
+        <v>26296</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>26821</v>
+        <v>26822</v>
       </c>
       <c r="I25" s="10" t="n">
-        <v>27357</v>
+        <v>27358</v>
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
@@ -17449,13 +17449,13 @@
         <v>68000</v>
       </c>
       <c r="G26" s="39" t="n">
-        <v>82068</v>
+        <v>82069</v>
       </c>
       <c r="H26" s="39" t="n">
-        <v>86959</v>
+        <v>86960</v>
       </c>
       <c r="I26" s="39" t="n">
-        <v>84904</v>
+        <v>84906</v>
       </c>
     </row>
     <row r="27">
@@ -17511,13 +17511,13 @@
         <v>131220.010876575</v>
       </c>
       <c r="G28" s="39" t="n">
-        <v>152068</v>
+        <v>152069</v>
       </c>
       <c r="H28" s="39" t="n">
-        <v>164959</v>
+        <v>164960</v>
       </c>
       <c r="I28" s="39" t="n">
-        <v>171904</v>
+        <v>171906</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Write GP margin (row6, Assumptions) as a literal value instead of a separate live formula
Previously Excel computed forecast GP margin via its own formula chain (referencing Q1 actual
GP/Revenue, 03_Revenue_Model!G2, and 17_Gia_Hang_Hoa spread cells), separate from the Python
gp_margin_fc variable already used for PDF/JSON - two independent implementations of the same
intended formula, prone to silent drift (confirmed via cell-by-cell comparison with the user's
open Excel file: P/B matched almost exactly, but EV/EBITDA and P/E differed by 6-12%, traced to
this GP margin divergence feeding into 04_PnL's EBIT/EBITDA/EPS chain).

Per user's request to stop maintaining two calculation paths: gp_margin_fc is now computed once
and written directly as Assumptions!G6/H6/I6, which 04_PnL's COGS/GP/EBIT formulas already
reference - so Excel, PDF, and JSON now all derive from the exact same number by construction.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/HPG/HPG_Model_2026_07_03.xlsx
+++ b/Bao cao/HPG/HPG_Model_2026_07_03.xlsx
@@ -2727,7 +2727,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>03/07/2026 18:20</t>
+          <t>03/07/2026 18:40</t>
         </is>
       </c>
     </row>
@@ -14051,17 +14051,14 @@
       <c r="F6" s="10" t="n">
         <v>15.69</v>
       </c>
-      <c r="G6" s="12">
-        <f>(G41+0.75*'03_Revenue_Model'!G2*(G41/G40)*(G47/G43))/'03_Revenue_Model'!G2*100</f>
-        <v/>
-      </c>
-      <c r="H6" s="12">
-        <f>G6*(G47/'17_Gia_Hang_Hoa'!G37)</f>
-        <v/>
-      </c>
-      <c r="I6" s="12">
-        <f>H6*(G47/'17_Gia_Hang_Hoa'!H37)</f>
-        <v/>
+      <c r="G6" s="12" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>12.8</v>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>

</xml_diff>